<commit_message>
Updated yield logic, alerts, reports
</commit_message>
<xml_diff>
--- a/data/employees.xlsx
+++ b/data/employees.xlsx
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
@@ -13033,13 +13033,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13344,13 +13346,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q656"/>
+  <dimension ref="A1:V656"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20" customWidth="1"/>
+    <col min="20" max="20" width="12" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="38.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -13403,7 +13409,7 @@
         <v>1932</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -13449,8 +13455,11 @@
       <c r="O2" t="s">
         <v>1269</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q2">
+        <v>9100001135187</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -13470,7 +13479,7 @@
         <v>1259</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -13490,7 +13499,7 @@
         <v>1259</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>632</v>
       </c>
@@ -13510,7 +13519,7 @@
         <v>1266</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -13530,7 +13539,7 @@
         <v>1261</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -13579,8 +13588,10 @@
       <c r="Q7">
         <v>21167045</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="T7" s="4"/>
+      <c r="V7" s="5"/>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -13630,7 +13641,7 @@
         <v>21171287</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -13680,7 +13691,7 @@
         <v>21167169</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -13730,7 +13741,7 @@
         <v>21216852</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -13780,7 +13791,7 @@
         <v>21199966</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -13830,7 +13841,7 @@
         <v>21154032</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -13880,7 +13891,7 @@
         <v>21195685</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -13930,7 +13941,7 @@
         <v>21175277</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -13974,7 +13985,7 @@
         <v>21181161</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>29</v>
       </c>

</xml_diff>